<commit_message>
docs(order-management): lock 24.15 scope — 8/8 deliverable, independent cron, settings-driven cadence (defaults pending BA), all ex-Blocked rows sequenced on 24.8
</commit_message>
<xml_diff>
--- a/order_management/24.15-payment-reminder-notifications/24.15 - Payment Reminder Notifications.xlsx
+++ b/order_management/24.15-payment-reminder-notifications/24.15 - Payment Reminder Notifications.xlsx
@@ -24,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,8 +43,12 @@
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -81,8 +85,13 @@
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -104,11 +113,25 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -147,6 +170,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -563,7 +595,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>8 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 0 out of scope.</t>
+          <t>SCOPE LOCKED at Step-1 gate 2026-07-03 (final story of the 7-story gate). 8/8 Deliverable — 5 sequenced intra-release on 24.8, 3 buildable now. Ship-together release; 24.15 builds LAST.</t>
         </is>
       </c>
     </row>
@@ -573,8 +605,10 @@
           <t>To implement here</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>8</v>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
@@ -585,13 +619,21 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>The story asks for an automatic, backend-enforced reminder system that nudges customers about upcoming and overdue payments and keeps nudging until an admin manually marks the installment "Paid" from the admin panel, at which point future reminders for that installment stop. Re-verification against the code confirms the notification DELIVERY machinery already exists and is proven: a NestJS @nestjs/schedule + SchedulerRegistry cron registrar pattern, a template-driven MailerService.sendFromTemplate that renders a NotificationTemplate, sends via SendGrid, and writes a NotificationLog — used today by low-balance/daily-summary/lead crons. However the story's central premise — a "manual payment" the customer pays outside Stripe and that an admin marks Paid — has NO write-path. The only installment ledger (PaymentTransaction) is exclusively a Stripe auto-charge ledger whose status is set to succeeded ONLY by the external-api webhook handler (and whose scheduled+due rows are auto-charged by the payment-charge cron, not reminded); CartPaymentScheduleEntry is explicitly "validation/display only — no charging happens here". No admin mark-as-Paid endpoint exists anywhere. So the reminder engine and templates are Deliverable as net-new on existing primitives, while the upcoming/overdue triggering, continuation, and stop-on-Paid logic are Blocked on the sibling Manual Payment Methods story.</t>
+          <t>Gate outcome: independent worker cron (D4a — not waiting for the unstarted E&amp;S scheduling system; hand-off note to the scheduling register), email-only (D1), settings-driven cadence (D2: payment_reminder_{upcoming_days,overdue_interval_days,hour_utc} = 7/7/14 pending BA — spec specifies NOTHING; gate directive: document provenance in code), manual-rows-only predicates mirroring the 24.8-D3 cron guard (disjoint partition), self-seeded slugs per the ownership rule, stop = PT.status read at send time (24.8 PATCH / 24.6 void) — no new state anywhere. All five former Blocked verdicts re-resolved to Deliverable-sequenced under the ship-together model.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr"/>
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Sequenced on 24.8</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>5 (a, b, e, f, g) — in-release, 24.8 builds first</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -610,7 +652,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -630,7 +672,7 @@
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -661,7 +703,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope locked 2026-07-03 (gate complete); plan after full 7-story gate</t>
         </is>
       </c>
     </row>
@@ -787,7 +829,7 @@
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>Impl Status (2026-07-01)</t>
+          <t>Impl Status (2026-07-03)</t>
         </is>
       </c>
     </row>
@@ -802,9 +844,9 @@
           <t>System shall automatically trigger reminder notifications to customers for UPCOMING payments.</t>
         </is>
       </c>
-      <c r="C2" s="10" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="C2" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.8)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -812,24 +854,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>The notification cron + send mechanism is buildable now, but there is no data source representing an 'upcoming payment the customer must pay manually'. The only installment model (PaymentTransaction, with due_date) is exclusively a Stripe off_session auto-charge ledger — the payment-charge cron charges these itself (WHERE status='scheduled' AND due_date&lt;=now()), so they are not 'awaiting customer payment'. CartPaymentScheduleEntry holds pre-order manual methods (check/wire/paypal) but is explicitly 'validation/display only — no charging happens here' and is not an order-level owed-payment record. The manual-payment installment lifecycle this requirement nudges on must be produced by the sibling Manual Payment Methods story.</t>
+          <t>Re-resolved from Blocked (ship-together release; 24.8 builds first). Cron mechanics always buildable ([status,due_date] index); the missing SEMANTIC — customer-actionable manual installment — is 24.8's payment_type column. Selection: status=scheduled AND payment_type != credit_card AND due_date &lt;= now()+upcoming_days — mirror image of the charge cron's 24.8-D3 guard, so the two crons partition rows disjointly by construction. D3 (interim predicate) RESOLVED-BY-SEQUENCING: 24.15 builds after 24.8, so the manual-rows predicate ships day one (no dark launch, no courtesy-email interim).</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:2056 (PaymentTransaction; due_date :2069; header comment confirms Stripe-only); admin-backend-api/prisma/schema.prisma:2838 (CartPaymentPlan 'validation/display only — no charging happens here'), :2853 (CartPaymentScheduleEntry); background-worker-service/src/jobs/payment-charge/payment-charge.service.ts:60 (chargeScheduled auto-charges scheduled+due rows)</t>
+          <t>PT :2073 (webhook-owned transitions), due_date :2086, index :2103; worker payment-charge.service.ts:60-67; 24.8 gate D2/D3 locked 2026-07-03</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Manual Payment Methods story (Order Management) — manual-payment installment lifecycle with an upcoming/awaiting-payment state</t>
+          <t>24.8 payment_type migration + cron guard — same release, builds first</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
@@ -845,7 +883,7 @@
       </c>
       <c r="L2" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story (Order Management) — manual-payment installment lifecycle with an upcoming/awaiting-payment state)</t>
+          <t>Gate 2026-07-03: Blocked -&gt; Deliverable-sequenced (D3 resolved-by-sequencing).</t>
         </is>
       </c>
     </row>
@@ -860,9 +898,9 @@
           <t>System shall automatically trigger reminder notifications to customers for OVERDUE payments.</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.8)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -870,24 +908,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Same gap as upcoming. 'Overdue' could in principle be derived from PaymentTransaction.due_date &lt; now AND status still scheduled, but those rows belong to the Stripe auto-charge flow (the cron charges them, it does not ask the customer to pay), and a failed Stripe installment goes to status=failed (auto-retried up to 3x), not to a manual-pay-overdue state. The PaymentTransactionStatus enum (scheduled/processing/succeeded/failed/canceled/refunded) has no manual-pay/overdue concept, and no code path writes a manual-payment 'overdue &amp; awaiting customer payment' record.</t>
+          <t>Re-resolved from Blocked. No stored 'overdue' — by design: mirror exhibitor deriveIsOverdue (due past AND status not in settled {succeeded,refunded,canceled}). Manual rows never cron-charged (24.8 guard) -&gt; overdue-manual = scheduled AND past-due AND payment_type != credit_card, repeating per overdue_interval_days w/ notification_logs dedupe. SUB-DECISION (option a, locked): retry-exhausted card rows (failed, retry_count=3) EXCLUDED — story is manual-framed; those rows already get the per-failure update-card email; BA may extend later (OQ-2).</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:491 (PaymentTransactionStatus enum — no manual-pay/overdue state); background-worker-service/src/jobs/payment-charge/payment-charge.service.ts:60 (scheduled+due rows are auto-charged, not reminded)</t>
+          <t>PaymentTransactionStatus :491-500 (no overdue value); MAX_AUTO_RETRIES=3 :18, retryFailed :74-82; exhibitor orders.helpers.ts:74-79 deriveIsOverdue, settled set :31</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Manual Payment Methods story (Order Management) — manual-payment overdue state</t>
+          <t>24.8 payment_type migration — same release</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr"/>
@@ -903,7 +937,7 @@
       </c>
       <c r="L3" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story (Order Management) — manual-payment overdue state)</t>
+          <t>Gate 2026-07-03: Blocked -&gt; Deliverable-sequenced (manual-only, option a).</t>
         </is>
       </c>
     </row>
@@ -918,7 +952,7 @@
           <t>Reminder delivery engine: send a templated notification to the customer via a backend scheduled job (cron).</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -928,19 +962,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E4" s="2" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Verified: the full delivery mechanism exists and is proven. @nestjs/schedule + SchedulerRegistry registrar pattern registers cron jobs (CronJob.from + registry.addCronJob); MailerService.sendFromTemplate renders a NotificationTemplate, sends via SendGrid, and appends a NotificationLog row (PENDING-&gt;SENT/FAILED). Low-balance/daily-summary/lead notification crons already follow exactly this cron-task -&gt; service -&gt; mailer shape. A new payment-reminder cron + service is net-new code on these built primitives. Caveat confirmed: only the EMAIL channel has a real dispatch path (SendGrid); SMS is only a NotificationChannel enum value with no send client.</t>
+          <t>Buildable NOW, independent of 24.8. D4a: INDEPENDENT worker cron (not waiting for the unstarted E&amp;S dynamic-scheduling system, which claims payment-due reminders — hand-off note filed in the SCHEDULING register per register-separation rule, OQ-4). Clone the payment-charge registrar/task pair (settings hours, CronJob.from + registry.addCronJob, per-kind overlap guard); reads the D2 settings family; dispatch via WORKER MailerService.sendFromTemplate (SendGrid; NotificationLog PENDING-&gt;SENT/FAILED). Worker has exactly 5 registrars, zero 'reminder' hits. MAILER SPLIT: cron leg = worker mailer; admin-triggered action emails (24.6-r/24.11/24.5) = admin's mailer; both write notification_logs — keep notification_type consistent.</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>background-worker-service/src/notification/mailer.service.ts:88 (sendFromTemplate; SendGrid import :5, NotificationLog audit :48); background-worker-service/src/notification/low-balance.service.ts:1 (proven cron-notification pattern); background-worker-service/src/scheduler/payment-charge/payment-charge-scheduler.registrar.ts:62-72 (CronJob.from + registry.addCronJob registration)</t>
+          <t>registrar :63-84 (hours :40-41, defaults 02:00/06:00); task :22/:32/:65; worker mailer.service.ts:88 (sgMail :5; log :48/:124/:160/:176); low-balance.service.ts precedent</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -961,7 +991,7 @@
       </c>
       <c r="L4" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable (D4a independent cron).</t>
         </is>
       </c>
     </row>
@@ -976,7 +1006,7 @@
           <t>Provide payment-reminder notification templates (upcoming + overdue) for the customer.</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -986,19 +1016,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Verified: the NotificationTemplate model (notification_type, channel EMAIL/SMS, tag, is_active, subject, body, tokens) plus the seeder pattern already supports adding new templated notifications. Today only a payment-RECEIPT template (notification_type 'ppl_product_order_payment', 'Order Payment Receipt') exists — no upcoming/overdue reminder template. Adding reminder templates is net-new seeding on built infra.</t>
+          <t>Buildable NOW. D1 EMAIL-ONLY (SendGrid is the only dispatch path; SMS = enum value w/ no client in any repo; enum accommodates SMS later w/o migration). D5 slugs payment_reminder_upcoming / payment_reminder_overdue, seeded BY 24.15 per the template-ownership rule (locked 24.11: flows own their templates; E&amp;S epic manages only). SBE-671 MERGED — unmerged-branch collision concern retired; dev's 29 trigger slugs have zero reminder entries (no collision). Placeholders from PT + order context (amount, due date, order number, method label via payment_type); copy at plan time, admin-editable after.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:237 (NotificationChannel enum EMAIL/SMS), :255 (NotificationTemplate model); admin-backend-api/src/database/seeds/notification-template.seeder.ts:138,578 (receipt template only; no reminder template)</t>
+          <t>NotificationTemplate :255; NotificationChannel :239-242; template seeder :142/:619 (receipt only); trigger-event seeder 29 slugs (verified 2026-07-03); SBE-671 merged PR#426</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1019,7 +1045,7 @@
       </c>
       <c r="L5" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable (D1 email-only; D5 self-seeded slugs).</t>
         </is>
       </c>
     </row>
@@ -1034,9 +1060,9 @@
           <t>Reminders shall CONTINUE (repeat) until the installment is marked Paid.</t>
         </is>
       </c>
-      <c r="C6" s="10" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.8)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -1044,24 +1070,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>A recurring cadence is buildable on the scheduler (the cron simply re-selects unpaid items each tick), but the termination predicate 'until marked Paid (manually)' has no readable signal. PaymentTransaction.status is only ever advanced to succeeded by the Stripe webhook handler; there is no manual 'Paid' state for a manual-payment installment for the cron to test against, so continuation cannot be correctly bounded.</t>
+          <t>Re-resolved from Blocked: NO NEW STATE — cron re-selects unpaid rows each tick and checks PT.status at send time; when 24.8's PATCH flips succeeded (or 24.6's void -&gt; canceled) the row drops out naturally. Dedupe-per-interval (D2) bounds 'continues' to the configured cadence. Recipient: billing_email per 24.11 chain; additional_emails CC pending consolidated OQ (with 24.6) — if ratified, one-line CC-append.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>external-api-service/src/modules/webhook/services/webhook.service.ts:738 (status set to succeeded only by webhook); admin-backend-api/prisma/schema.prisma:491 (no manual-paid state); grep of admin-backend-api/src for markPaid/record-payment/mark-installment returned no write path</t>
+          <t>webhook.service.ts:738 (current sole succeeded writer); no installment write-path on dev (re-grepped 2026-07-03); 24.8-c locked semantics</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Manual Payment Methods story (Order Management) — a Paid state writable from the admin panel</t>
+          <t>24.8 installment PATCH — same release</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
@@ -1077,7 +1099,7 @@
       </c>
       <c r="L6" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story (Order Management) — a Paid state writable from the admin panel)</t>
+          <t>Gate 2026-07-03: Blocked -&gt; Deliverable-sequenced (no new state; recipient locked).</t>
         </is>
       </c>
     </row>
@@ -1092,9 +1114,9 @@
           <t>Stop condition: once the admin marks the installment Paid from the admin panel, all future reminders for that installment stop automatically.</t>
         </is>
       </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="C7" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.8)</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -1102,24 +1124,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Verified absent: there is no admin endpoint or any code path that marks an installment/payment Paid. The PaymentTransaction status is flipped to succeeded solely by the Stripe webhook handler (and source enum 'manual_retry' is still a Stripe retry, not a manual cash/check settlement). The admin-backend-api has no manual mark-as-Paid mutation for installments (no controller writes PaymentTransaction). Without that admin write-path the stop signal does not exist; this capability is owned by the Manual Payment Methods story.</t>
+          <t>Re-resolved from Blocked: mark-as-Paid = 24.8's PATCH :id/payment-plan/installments/:installmentId (locked at its gate: manual-method-only, Paid -&gt; succeeded). Stop check is the SAME status read as 24.15-e — same build; works the day 24.8 ships (before 24.15 in release order). Evidence refresh: PaymentTransactionSource now 6 values (+admin_change_plan, +admin_manual per 24.8-D4) — no exhaustive switch may assume fewer.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>external-api-service/src/modules/webhook/services/webhook.service.ts:738 (webhook is sole writer of succeeded); admin-backend-api/prisma/schema.prisma:503 (PaymentTransactionSource: checkout/cron/manual_retry/subscription_renewal — all Stripe); grep across admin/external/exhibitor/worker src found no mark-paid installment write-path</t>
+          <t>24.8 doc 24.8-c/D4 locked 2026-07-03; PaymentTransactionSource :503-511 (6 values)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Manual Payment Methods story (Order Management) — admin 'mark installment Paid' write-path</t>
+          <t>24.8 installment PATCH — same release</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -1135,7 +1153,7 @@
       </c>
       <c r="L7" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story (Order Management) — admin 'mark installment Paid' write-path)</t>
+          <t>Gate 2026-07-03: Blocked -&gt; Deliverable-sequenced (+ source-enum refresh).</t>
         </is>
       </c>
     </row>
@@ -1150,9 +1168,9 @@
           <t>Reminder scheduling AND stop logic shall be enforced on the backend (not the client).</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Blocked</t>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>Deliverable — sequenced intra-release (24.8)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -1160,24 +1178,20 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>The scheduling half is naturally backend-enforceable (cron in background-worker-service, no client involvement) and would be Deliverable on its own. But the stop-logic half cannot be enforced because the 'Paid' state it must read is never written (see 24.15-f), and the trigger set it must schedule on does not exist (see 24.15-a/b). Since the combined backend rule cannot be correctly enforced now, it is Blocked on the same Manual Payment Methods dependency.</t>
+          <t>Re-resolved from Blocked: scheduling half = worker cron (no client involvement by construction); stop half = e/f status check, sequenced on 24.8. CORRECTION from later gates: 24.7's order-level PATCH :id/payment-status (the old 'secondary stop signal') was DROPPED at the 24.7 gate — stop signals are exactly 24.8's PATCH (succeeded) and 24.6's void (canceled), both covered by the settled-set check without special-casing.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>background-worker-service/src/scheduler/payment-charge/payment-charge-scheduler.registrar.ts:62-72 (backend cron framework exists); external-api-service/src/modules/webhook/services/webhook.service.ts:738 (paid only via webhook, no manual stop signal)</t>
+          <t>registrar refs (24.15-c); 24.7 doc D3 (PATCH dropped, locked 2026-07-03)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Manual Payment Methods story (Order Management) — manual Paid state + manual-payment trigger source</t>
+          <t>24.8 (stop half) — same release</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -1193,7 +1207,7 @@
       </c>
       <c r="L8" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story (Order Management) — manual Paid state + manual-payment trigger source)</t>
+          <t>Gate 2026-07-03: Blocked -&gt; Deliverable-sequenced (24.7 correction folded in).</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1222,7 @@
           <t>No dedicated screen — the feature is purely an automatic backend behavior with no UI.</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" s="1" t="inlineStr">
         <is>
           <t>Deliverable</t>
         </is>
@@ -1218,19 +1232,15 @@
           <t>Implement here</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Design constraint, honored trivially by implementing this as a background cron only (no controller/screen). Consistent with existing UI-less notification crons (low-balance, daily-summary). Nothing to build beyond respecting the constraint; an optional dev-only manual-trigger endpoint mirrors the existing precedent.</t>
+          <t>Buildable NOW. Cron-only + one dev-only POST manual-trigger/payment-reminders/run (controller has exactly the lead-distribution + low-balance precedents). Nav-clause tension ('System, payment reminders' breadcrumb vs UI-less Design Spec) resolved cheaply by D2: the settings family IS the future config surface if BA ever wants one; flagged in OQ-1.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>background-worker-service/src/notification/low-balance.service.ts:1 (UI-less notification cron precedent); background-worker-service/src/manual-trigger/manual-trigger.controller.ts:55 (dev-only @Post('low-balance/run') precedent, no customer/admin UI)</t>
+          <t>manual-trigger.controller.ts :17/:26/:55 (only 2 handlers today)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1247,7 +1257,7 @@
       </c>
       <c r="L9" s="12" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Gate 2026-07-03: Deliverable.</t>
         </is>
       </c>
     </row>
@@ -1273,7 +1283,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1311,29 +1321,56 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>POST</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="14" t="inlineStr">
         <is>
           <t>background-worker-service: /manual-trigger/payment-reminders/run</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Dev-only manual trigger to invoke the payment-reminder cron on demand (reuses task.run()). The reminder itself runs on a registered cron; no customer- or admin-facing REST/UI endpoint.</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>24.15-c, 24.15-e, 24.15-g</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Depends on the 24.8 mark-as-Paid capability (PATCH .../installments/:installmentId) for its stop condition.</t>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Dev-only manual trigger invoking the reminder task on demand (mirrors low-balance/lead precedents). The feature itself is a registered cron — no customer/admin REST or UI endpoint.</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>24.15-c, e, g, h</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Stop condition reads statuses written by 24.8's PATCH + 24.6's void</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>(settings)</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>payment_reminder_upcoming_days / payment_reminder_overdue_interval_days / payment_reminder_hour_utc</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>ppl-settings family (defaults 7 / 7 / 14 UTC pending BA ratification, OQ-1) with gate-provenance doc-comments per the D2 directive — the spec contains NO cadence/window/hour anywhere.</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>24.15-a, b, e</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Mirrors payment_charge_hour_utc family</t>
         </is>
       </c>
     </row>
@@ -1348,74 +1385,252 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
-    <col width="34" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="9" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="9" t="inlineStr">
-        <is>
-          <t>Open Question</t>
-        </is>
-      </c>
-      <c r="C1" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D1" s="9" t="inlineStr">
-        <is>
-          <t>Resolution / Decision</t>
+      <c r="B1" s="15" t="inlineStr">
+        <is>
+          <t>Req</t>
+        </is>
+      </c>
+      <c r="C1" s="15" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D1" s="15" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+      <c r="E1" s="15" t="inlineStr">
+        <is>
+          <t>Open Question / What is needed</t>
+        </is>
+      </c>
+      <c r="F1" s="15" t="inlineStr">
+        <is>
+          <t>Dependency (blocking story + Jira)</t>
+        </is>
+      </c>
+      <c r="G1" s="15" t="inlineStr">
+        <is>
+          <t>Assignee</t>
+        </is>
+      </c>
+      <c r="H1" s="15" t="inlineStr">
+        <is>
+          <t>Sprint / Jira status</t>
+        </is>
+      </c>
+      <c r="I1" s="15" t="inlineStr">
+        <is>
+          <t>Decision / Current direction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Channel scope: the spec says 'reminder notifications to customers' without naming a channel. Only EMAIL has a real dispatch path (SendGrid); SMS exists only as a NotificationChannel enum value with no send client. Is email-only acceptable, or is SMS in scope (which would require a net-new SMS provider integration)?</t>
-        </is>
-      </c>
-      <c r="C2" s="12" t="inlineStr">
-        <is>
-          <t>[OPEN — for team discussion]</t>
-        </is>
-      </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): lean email-only for the first cut (EMAIL is the only channel with a proven SendGrid dispatch path; SMS would require a net-new provider integration) — pending team confirmation.</t>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>OQ-1</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>24.15-a/b/e (D2)</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Cadence defaults ratification + nav clause</t>
+        </is>
+      </c>
+      <c r="D2" s="14" t="inlineStr">
+        <is>
+          <t>Deliverable (mechanism locked)</t>
+        </is>
+      </c>
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Ratify proposed defaults: upcoming 7 days before due (single send); overdue every 7 days after due until settled; send hour 14:00 UTC. Values exist NOWHERE in the spec — set at the 2026-07-03 gate; settings-driven so BA's answer changes a seeded default, not code. Also: does the 'System, payment reminders' nav breadcrumb imply a cadence-config screen? (Build is UI-less per 24.15-h; the settings family is the natural surface if yes.)</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>Open 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Build proceeds on defaults; code doc-comments state provenance + pending ratification (gate directive).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Reminder cadence is unspecified: how many reminders, and at what intervals before due (upcoming) and after due (overdue)?</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>[OPEN — for team discussion]</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Current direction (2026-07-01): (pending) — the number of reminders and the before-/after-due intervals must be defined by the team before the cron schedule can be written.</t>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>OQ-2</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>24.15-b</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Retry-exhausted card rows excluded</t>
+        </is>
+      </c>
+      <c r="D3" s="14" t="inlineStr">
+        <is>
+          <t>Deliverable (manual-only locked)</t>
+        </is>
+      </c>
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Overdue reminders select MANUAL rows only. Stuck card rows (failed, retry_count=3, abandoned by retry cron) are customer-actionable but excluded — they already get the per-failure update-card email. BA may extend the predicate later (small change: widen the status/type filter).</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>Open 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>Option (a) locked; extension is a predicate tweak, not a redesign.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>OQ-3</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>24.15-e (recipient)</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>additional_emails CC scope</t>
+        </is>
+      </c>
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>Deliverable (to = billing_email locked)</t>
+        </is>
+      </c>
+      <c r="E4" s="14" t="inlineStr">
+        <is>
+          <t>Consolidated with 24.6's OQ-2 — ONE BA answer for all four senders (24.6-r, 24.11, 24.15, 24.5). If ratified: one-line CC-append in this cron's dispatch.</t>
+        </is>
+      </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G4" s="14" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="H4" s="14" t="inlineStr">
+        <is>
+          <t>Open 2026-07-03</t>
+        </is>
+      </c>
+      <c r="I4" s="14" t="inlineStr">
+        <is>
+          <t>Reminders go to billing_email until answered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>OQ-4</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>24.15-c (D4)</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="inlineStr">
+        <is>
+          <t>Scheduling-system hand-off</t>
+        </is>
+      </c>
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>Deliverable (independent cron locked)</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
+        <is>
+          <t>E&amp;S dynamic-scheduling design (implementation not started) claims payment-due reminders (ANCHOR_RELATIVE). 24.15 ships independent; the future scheduling build must absorb or knowingly coexist with this cron. Hand-off note to be filed in the SCHEDULING known-issues register (per register-separation rule — NOT the main E&amp;S register) when 24.15 ships.</t>
+        </is>
+      </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>E&amp;S scheduling implementation (unstarted; own doc set)</t>
+        </is>
+      </c>
+      <c r="G5" s="14" t="inlineStr">
+        <is>
+          <t>— (recorded for the scheduling effort)</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>Design done, build not started</t>
+        </is>
+      </c>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>D4a locked: ship now, migrate later.</t>
         </is>
       </c>
     </row>
@@ -1430,7 +1645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="55" customWidth="1" min="1" max="1"/>
@@ -1456,36 +1671,53 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>A manual-payment installment lifecycle — installments paid outside Stripe (check / bank wire / paypal) that carry an 'awaiting payment / upcoming / overdue' state distinct from the Stripe auto-charge PaymentTransaction flow. Reminders have nothing to act on without it.</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>24.15-a, 24.15-b, 24.15-e, 24.15-g</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Order Management — Manual Payment Methods story (sibling, not yet built)</t>
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>In-release (NOT external): 24.8 payment_type migration + cron guard + installment PATCH (SBE-1132) — manual lifecycle, selection column, stop signal</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>24.15-a, b, e, f, g</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="inlineStr">
+        <is>
+          <t>Same release — 24.8 builds first; 24.15 builds last</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>An admin 'mark installment Paid' write-path from the admin panel that sets a Paid status the reminder cron can read. Today PaymentTransaction.status is set to succeeded only by the Stripe webhook; no manual mark-as-Paid endpoint exists in any repo.</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>24.15-f, 24.15-e, 24.15-g</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Order Management — Manual Payment Methods story (sibling, not yet built)</t>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>In-release: 24.6 void endpoint (canceled rows drop out via the settled-set check)</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>24.15-e/f stop coverage</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr">
+        <is>
+          <t>Same release (24.6, D-z)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="14" t="inlineStr">
+        <is>
+          <t>E&amp;S dynamic-scheduling system (future) — absorbs/supersedes this cron per OQ-4 hand-off</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>post-release migration only</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="inlineStr">
+        <is>
+          <t>E&amp;S scheduling effort (docs done, build unstarted)</t>
         </is>
       </c>
     </row>
@@ -1500,7 +1732,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1520,194 +1752,158 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
-        <is>
-          <t>Not started — analysis/feasibility stage only; no branch or SBE ticket cut yet.</t>
+      <c r="B2" s="14" t="inlineStr">
+        <is>
+          <t>Not started — Step-1 gate complete 2026-07-03 (8-item walkthrough with Prantik; FINAL story of the 7-story gate). Scope locked: 8/8 Deliverable — 5 sequenced intra-release on 24.8 (a,b,e,f,g), 3 independently buildable (c,d,h). Release model: ship-together; 24.15 builds LAST.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>Branch / Commits / PR</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>— (not started). No SBE ticket / PR / Swagger tag yet.</t>
+      <c r="A3" s="16" t="inlineStr">
+        <is>
+          <t>Branch</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-a</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story) — upcoming-payment reminder trigger; no manual-payment upcoming/awaiting-payment data source.</t>
+      <c r="A4" s="16" t="inlineStr">
+        <is>
+          <t>SBE ticket</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr">
+        <is>
+          <t>SBE-1139 (In Progress, Prantik Saha)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-b</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story) — overdue-payment reminder trigger; no manual-pay overdue/awaiting record.</t>
+      <c r="A5" s="16" t="inlineStr">
+        <is>
+          <t>Commits</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-c</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — reminder delivery engine (net-new cron + service over the proven MailerService.sendFromTemplate primitives).</t>
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-d</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — reminder templates (upcoming + overdue); net-new seeding on the built NotificationTemplate infra.</t>
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Swagger tag</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-e</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story) — reminders continue until Paid; termination predicate has no readable manual-Paid signal.</t>
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Build gates</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-f</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story) — stop once admin marks Paid; no admin mark-as-Paid write-path exists.</t>
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>Live smoke</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-g</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started (Blocked — Manual Payment Methods story) — backend-enforced scheduling + stop; scheduling half OK, stop half blocked.</t>
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Confirmed build scope</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr">
+        <is>
+          <t>Independent worker cron (clone payment-charge registrar/task pair) + selection predicates (upcoming/overdue, manual rows only via payment_type) + 2 EMAIL templates + slugs payment_reminder_upcoming/overdue (self-seeded) + 3 ppl-settings knobs (7/7/14 defaults, gate-provenance doc-comments REQUIRED) + notification_logs dedupe + dev-only manual trigger. Recipient = billing_email.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>Not started — 24.15-h</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>◻ Not started — no dedicated screen; honored by building a background cron only (no controller/screen).</t>
+      <c r="A11" s="16" t="inlineStr">
+        <is>
+          <t>Decisions</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>D1 email-only · D2 settings mechanism (values pending BA, OQ-1) · D3 resolved-by-sequencing · D4a independent cron (hand-off OQ-4) · D5 self-seeded slugs · 24.15-b manual-only (OQ-2)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>Remaining in story</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>All in-scope requirements remain: 24.15-a, 24.15-b, 24.15-c, 24.15-d, 24.15-e, 24.15-f, 24.15-g, 24.15-h.</t>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>External dependencies — see Cross-Epic Dependencies</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>None external; in-release: 24.8 (builds first) + 24.6 void</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>Open decision — Channel scope</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Email-only vs SMS in scope (SMS would require a net-new provider integration) — pending team confirmation.</t>
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Out of API scope</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr">
+        <is>
+          <t>FE anything (story is UI-less); SMS channel (D1 — enum-ready, no client)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>Open decision — Reminder cadence</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>How many reminders, and at what intervals before due (upcoming) / after due (overdue) — (pending).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>Dependency — Manual Payment Methods story</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Manual-payment installment lifecycle (upcoming/awaiting/overdue state) — needed for 24.15-a, 24.15-b, 24.15-e, 24.15-g. (owner: Order Management, sibling, not yet built)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>Dependency — Manual Payment Methods story</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>Admin 'mark installment Paid' write-path (Paid status the reminder cron can read) — needed for 24.15-f, 24.15-e, 24.15-g. (owner: Order Management, sibling, not yet built)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Out of API scope</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>Front-end wiring is outside API scope; there is no Out-of-Scope requirement in this story.</t>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>Evidence baseline</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Verified @admin 0ac2769 (+4 siblings) 2026-07-03; line-drift corrections applied (PT :2073, seeder :142/:619, registrar :63-84, source enum 6 values); dev same-day move to 34c6fb4 does not touch this story's evidence.</t>
         </is>
       </c>
     </row>

</xml_diff>